<commit_message>
Admin File is still sucks
</commit_message>
<xml_diff>
--- a/server/uploads/admin-data.xlsx
+++ b/server/uploads/admin-data.xlsx
@@ -40,25 +40,25 @@
     <t>Last Updated</t>
   </si>
   <si>
-    <t>236540307054</t>
-  </si>
-  <si>
-    <t>Hely Patel</t>
-  </si>
-  <si>
-    <t>helykikani2020@gmail.com</t>
-  </si>
-  <si>
-    <t>Diploma</t>
+    <t>236540307057</t>
+  </si>
+  <si>
+    <t>Helu</t>
+  </si>
+  <si>
+    <t>helykikani0209@gmail.com</t>
+  </si>
+  <si>
+    <t>B.Sc</t>
   </si>
   <si>
     <t>Computer</t>
   </si>
   <si>
-    <t>85</t>
-  </si>
-  <si>
-    <t>2566264154</t>
+    <t>87</t>
+  </si>
+  <si>
+    <t>1236547825</t>
   </si>
   <si>
     <t>10/19/2025</t>
@@ -496,7 +496,7 @@
         <v>13</v>
       </c>
       <c r="F2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G2" t="s">
         <v>14</v>

</xml_diff>